<commit_message>
WORKFLOW MODIFIED FOR git actions
</commit_message>
<xml_diff>
--- a/north_india_deep_contacts.xlsx
+++ b/north_india_deep_contacts.xlsx
@@ -509,14 +509,10 @@
           <t>https://www.abhilashiuniversity.ac.in/Placement-cell, https://www.abhilashiuniversity.ac.in/Career</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>registrar@abhilashiuniversity.ac.in, regabhilashi@gmail.com</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1907292607, +91-8278845894, 1907292611, 9459052533, +91-9418453239, 01907292611, 1907250405, +91-9459052533, +91-9816242139, 9418453239, 01907292607, 01907250405, 8278845894, 9816242139, +919418453239</t>
+          <t>9418453239, 1907250405, 1907292611, 9816242139, 9459052533, 8278845894, 1907292607</t>
         </is>
       </c>
     </row>
@@ -612,7 +608,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>93023-93023, 9302393023, 1645055172, 0164-5055100, 1645055255, 01645055000, 1645055000, 0164-5055045, 1645055100, 0164-5055000, 1645055045, 0164-5055172, 1645055208</t>
+          <t>1645055045, 1645055100, 0164-5055172, 01645055000, 0164-5055000, 1645055000, 1645055208, 0164-5055100, 1645055255, 93023-93023, 1645055172, 0164-5055045, 9302393023</t>
         </is>
       </c>
     </row>
@@ -670,7 +666,11 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0129-2400605</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>